<commit_message>
Tie QA defects to use cases and document missing diagram
</commit_message>
<xml_diff>
--- a/outputs/iteration-2/iteration-2-bug-report.xlsx
+++ b/outputs/iteration-2/iteration-2-bug-report.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Summary" sheetId="1" r:id="R467dcd5e670d4f2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Details" sheetId="2" r:id="R9034ef433b2e4b13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Summary" sheetId="1" r:id="Ra17172d529a24bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Details" sheetId="2" r:id="R2eae2bb917ee4798"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -481,7 +481,7 @@
     </x:row>
     <x:row r="2" ht="85" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>BUG-001</x:v>
+        <x:v>UC-002-BUG-001</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
         <x:v>TC-008R; TC-009 blocked</x:v>
@@ -531,7 +531,7 @@
     </x:row>
     <x:row r="3" ht="85" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>BUG-002</x:v>
+        <x:v>UC-003-BUG-001</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
         <x:v>TC-010; TC-011</x:v>
@@ -581,7 +581,7 @@
     </x:row>
     <x:row r="4" ht="85" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>BUG-003</x:v>
+        <x:v>UC-003-BUG-002</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
         <x:v>TC-012</x:v>
@@ -631,7 +631,7 @@
     </x:row>
     <x:row r="5" ht="85" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>BUG-004</x:v>
+        <x:v>UC-002-BUG-002</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
         <x:v>TC-014</x:v>
@@ -681,7 +681,7 @@
     </x:row>
     <x:row r="6" ht="85" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>BUG-006</x:v>
+        <x:v>UC-001-BUG-001</x:v>
       </x:c>
       <x:c r="B6" s="2" t="str">
         <x:v>TC-015</x:v>
@@ -731,7 +731,7 @@
     </x:row>
     <x:row r="7" ht="85" customHeight="1">
       <x:c r="A7" s="2" t="str">
-        <x:v>BUG-007</x:v>
+        <x:v>SETUP-BUG-001</x:v>
       </x:c>
       <x:c r="B7" s="2" t="str">
         <x:v>TC-018</x:v>
@@ -781,7 +781,7 @@
     </x:row>
     <x:row r="8" ht="85" customHeight="1">
       <x:c r="A8" s="2" t="str">
-        <x:v>BUG-008</x:v>
+        <x:v>UC-004-BUG-001</x:v>
       </x:c>
       <x:c r="B8" s="2" t="str">
         <x:v>TC-016</x:v>

</xml_diff>